<commit_message>
vault backup: 2026-09-21 19:40:00
</commit_message>
<xml_diff>
--- a/01-Projects/에이팜건강-주간자금계획-자동화/자금계획_자동화/03_은행거래내역/우리은행/우리은행 거래내역조회 20260921.xlsx
+++ b/01-Projects/에이팜건강-주간자금계획-자동화/자금계획_자동화/03_은행거래내역/우리은행/우리은행 거래내역조회 20260921.xlsx
@@ -1,10 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr codeName="ThisWorkbook"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\AP\Documents\mynotes\01-Projects\에이팜건강-주간자금계획-자동화\자금계획_자동화\03_은행거래내역\우리은행\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{32BFC6BA-771F-4109-A662-F55E94F9E238}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
     <sheet name="Sheet" sheetId="1" r:id="rId1"/>
   </sheets>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
@@ -80,7 +91,7 @@
     <t>2026.09.21 05:14:42</t>
   </si>
   <si>
-    <t xml:space="preserve">펌뱅킹　</t>
+    <t>펌뱅킹　</t>
   </si>
   <si>
     <t>스마트스토어정산</t>
@@ -131,9 +142,9 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x14ac">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="165" formatCode="0_ "/>
+    <numFmt numFmtId="176" formatCode="0_ "/>
   </numFmts>
   <fonts count="12" x14ac:knownFonts="1">
     <font>
@@ -141,143 +152,140 @@
       <name val="Calibri"/>
     </font>
     <font>
+      <b/>
       <sz val="12"/>
-      <name val="Calibri"/>
+      <color rgb="FF000000"/>
+      <name val="맑은 고딕"/>
+      <family val="3"/>
+      <charset val="129"/>
     </font>
     <font>
+      <b/>
       <sz val="12"/>
+      <color rgb="FF000000"/>
       <name val="맑은 고딕"/>
-      <b/>
-      <color rgb="#000000"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <name val="맑은 고딕"/>
-      <b/>
-      <color rgb="#000000"/>
+      <family val="3"/>
+      <charset val="129"/>
     </font>
     <font>
       <sz val="10"/>
+      <color rgb="FF000000"/>
       <name val="Arial"/>
-      <color rgb="#000000"/>
     </font>
     <font>
       <sz val="10"/>
+      <color rgb="FF000000"/>
       <name val="Arial"/>
-      <color rgb="#000000"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FF707070"/>
+      <name val="맑은 고딕"/>
+      <family val="3"/>
+      <charset val="129"/>
     </font>
     <font>
       <sz val="10"/>
+      <color rgb="FF000000"/>
       <name val="맑은 고딕"/>
-      <b/>
-      <color rgb="FF707070"/>
+      <family val="3"/>
+      <charset val="129"/>
     </font>
     <font>
       <sz val="10"/>
+      <color rgb="FF000000"/>
       <name val="맑은 고딕"/>
-      <color rgb="#000000"/>
+      <family val="3"/>
+      <charset val="129"/>
     </font>
     <font>
       <sz val="10"/>
+      <color rgb="FF000000"/>
       <name val="맑은 고딕"/>
-      <color rgb="#000000"/>
+      <family val="3"/>
+      <charset val="129"/>
     </font>
     <font>
       <sz val="10"/>
+      <color rgb="FF000000"/>
       <name val="맑은 고딕"/>
-      <color rgb="#000000"/>
+      <family val="3"/>
+      <charset val="129"/>
     </font>
     <font>
       <sz val="10"/>
+      <color rgb="FF000000"/>
       <name val="맑은 고딕"/>
-      <color rgb="#000000"/>
+      <family val="3"/>
+      <charset val="129"/>
     </font>
     <font>
-      <sz val="10"/>
-      <name val="맑은 고딕"/>
-      <color rgb="#000000"/>
+      <sz val="8"/>
+      <name val="돋움"/>
+      <family val="3"/>
+      <charset val="129"/>
     </font>
   </fonts>
   <fills count="12">
     <fill>
-      <patternFill patternType="none">
-        <bgColor/>
-      </patternFill>
+      <patternFill patternType="none"/>
     </fill>
     <fill>
-      <patternFill patternType="gray125">
-        <bgColor/>
+      <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="none">
+        <fgColor rgb="FF000000"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="none">
         <fgColor rgb="FF000000"/>
-        <bgColor/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="none">
         <fgColor rgb="FF000000"/>
-        <bgColor/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="none">
         <fgColor rgb="FF000000"/>
-        <bgColor/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF8F8F8"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="none">
         <fgColor rgb="FF000000"/>
-        <bgColor/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFf8f8f8"/>
-        <bgColor/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="none">
         <fgColor rgb="FF000000"/>
-        <bgColor/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="none">
         <fgColor rgb="FF000000"/>
-        <bgColor/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="none">
         <fgColor rgb="FF000000"/>
-        <bgColor/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="none">
         <fgColor rgb="FF000000"/>
-        <bgColor/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="none">
-        <fgColor rgb="FF000000"/>
-        <bgColor/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="10">
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
+  <borders count="9">
     <border>
       <left/>
       <right/>
@@ -406,49 +414,55 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs>
+  <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="1" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="49" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="5" fillId="6" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="176" fontId="6" fillId="7" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="4" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="8" fillId="9" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="9" fillId="10" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="10" fillId="11" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="5" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="4" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="6" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="7" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="8" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="9" fillId="9" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="10" fillId="10" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="11" fillId="11" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
   </cellXfs>
-  <cellStyles>
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+  <cellStyles count="1">
+    <cellStyle name="표준" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -773,435 +787,433 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Sheet"/>
   <dimension ref="A1:J13"/>
+  <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="7.50390625" customWidth="1"/>
-    <col min="2" max="2" width="20.75390625" customWidth="1"/>
-    <col min="3" max="3" width="12.50390625" customWidth="1"/>
+    <col min="1" max="1" width="7.5" customWidth="1"/>
+    <col min="2" max="2" width="20.75" customWidth="1"/>
+    <col min="3" max="3" width="12.5" customWidth="1"/>
     <col min="4" max="4" width="18.375" customWidth="1"/>
-    <col min="5" max="5" width="18.75390625" customWidth="1"/>
-    <col min="6" max="6" width="18.75390625" customWidth="1"/>
-    <col min="7" max="7" width="18.75390625" customWidth="1"/>
-    <col min="8" max="8" width="16.375" customWidth="1"/>
-    <col min="9" max="9" width="16.375" customWidth="1"/>
-    <col min="10" max="10" width="18.75390625" customWidth="1"/>
+    <col min="5" max="7" width="18.75" customWidth="1"/>
+    <col min="8" max="9" width="16.375" customWidth="1"/>
+    <col min="10" max="10" width="18.75" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="4" t="s">
-        <v>0</v>
-      </c>
-      <c r="C1" s="4" t="s">
-        <v>0</v>
-      </c>
-      <c r="D1" s="4" t="s">
-        <v>0</v>
-      </c>
-      <c r="E1" s="4" t="s">
-        <v>0</v>
-      </c>
-      <c r="F1" s="4" t="s">
-        <v>0</v>
-      </c>
-      <c r="G1" s="4" t="s">
-        <v>0</v>
-      </c>
-      <c r="H1" s="4" t="s">
-        <v>0</v>
-      </c>
-      <c r="I1" s="4" t="s">
-        <v>0</v>
-      </c>
-      <c r="J1" s="4" t="s">
+    <row r="1" spans="1:10" ht="17.25" x14ac:dyDescent="0.25">
+      <c r="A1" s="7" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="8" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="8" t="s">
+        <v>0</v>
+      </c>
+      <c r="D1" s="8" t="s">
+        <v>0</v>
+      </c>
+      <c r="E1" s="8" t="s">
+        <v>0</v>
+      </c>
+      <c r="F1" s="8" t="s">
+        <v>0</v>
+      </c>
+      <c r="G1" s="8" t="s">
+        <v>0</v>
+      </c>
+      <c r="H1" s="8" t="s">
+        <v>0</v>
+      </c>
+      <c r="I1" s="8" t="s">
+        <v>0</v>
+      </c>
+      <c r="J1" s="8" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="5" t="s">
+    <row r="2" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A2" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="6" t="s">
+      <c r="B2" s="10" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="6" t="s">
+      <c r="C2" s="10" t="s">
         <v>1</v>
       </c>
-      <c r="D2" s="6" t="s">
+      <c r="D2" s="10" t="s">
         <v>1</v>
       </c>
-      <c r="E2" s="6" t="s">
+      <c r="E2" s="10" t="s">
         <v>1</v>
       </c>
-      <c r="F2" s="6" t="s">
+      <c r="F2" s="10" t="s">
         <v>1</v>
       </c>
-      <c r="G2" s="6" t="s">
+      <c r="G2" s="10" t="s">
         <v>1</v>
       </c>
-      <c r="H2" s="6" t="s">
+      <c r="H2" s="10" t="s">
         <v>1</v>
       </c>
-      <c r="I2" s="6" t="s">
+      <c r="I2" s="10" t="s">
         <v>1</v>
       </c>
-      <c r="J2" s="6" t="s">
+      <c r="J2" s="10" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="6" t="s">
+    <row r="3" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A3" s="10" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="6" t="s">
+      <c r="B3" s="10" t="s">
         <v>2</v>
       </c>
-      <c r="C3" s="6" t="s">
+      <c r="C3" s="10" t="s">
         <v>2</v>
       </c>
-      <c r="D3" s="6" t="s">
+      <c r="D3" s="10" t="s">
         <v>2</v>
       </c>
-      <c r="E3" s="6" t="s">
+      <c r="E3" s="10" t="s">
         <v>2</v>
       </c>
-      <c r="F3" s="6" t="s">
+      <c r="F3" s="10" t="s">
         <v>2</v>
       </c>
-      <c r="G3" s="6" t="s">
+      <c r="G3" s="10" t="s">
         <v>2</v>
       </c>
-      <c r="H3" s="6" t="s">
+      <c r="H3" s="10" t="s">
         <v>2</v>
       </c>
-      <c r="I3" s="6" t="s">
+      <c r="I3" s="10" t="s">
         <v>2</v>
       </c>
-      <c r="J3" s="6" t="s">
+      <c r="J3" s="10" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="7" t="s">
+    <row r="4" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="7" t="s">
+      <c r="B4" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="C4" s="7" t="s">
+      <c r="C4" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="D4" s="7" t="s">
+      <c r="D4" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="E4" s="7" t="s">
+      <c r="E4" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="F4" s="7" t="s">
+      <c r="F4" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="G4" s="7" t="s">
+      <c r="G4" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="H4" s="7" t="s">
+      <c r="H4" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="I4" s="7" t="s">
+      <c r="I4" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="J4" s="7" t="s">
+      <c r="J4" s="1" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="8">
+    <row r="5" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A5" s="2">
         <v>1</v>
       </c>
-      <c r="B5" s="9" t="s">
+      <c r="B5" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="C5" s="9" t="s">
+      <c r="C5" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="D5" s="10" t="s">
+      <c r="D5" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="E5" s="11">
+      <c r="E5" s="5">
         <v>632250</v>
       </c>
-      <c r="F5" s="11">
-        <v>0</v>
-      </c>
-      <c r="G5" s="11">
+      <c r="F5" s="5">
+        <v>0</v>
+      </c>
+      <c r="G5" s="5">
         <v>14174014</v>
       </c>
-      <c r="H5" s="9" t="s">
+      <c r="H5" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="I5" s="10" t="s">
+      <c r="I5" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="J5" s="11">
+      <c r="J5" s="5">
         <v>0</v>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="8">
+    <row r="6" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A6" s="2">
         <v>2</v>
       </c>
-      <c r="B6" s="9" t="s">
+      <c r="B6" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="C6" s="9" t="s">
+      <c r="C6" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="D6" s="10" t="s">
+      <c r="D6" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="E6" s="11">
+      <c r="E6" s="5">
         <v>330000</v>
       </c>
-      <c r="F6" s="11">
-        <v>0</v>
-      </c>
-      <c r="G6" s="11">
+      <c r="F6" s="5">
+        <v>0</v>
+      </c>
+      <c r="G6" s="5">
         <v>14806264</v>
       </c>
-      <c r="H6" s="9" t="s">
+      <c r="H6" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="I6" s="10" t="s">
+      <c r="I6" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="J6" s="11">
+      <c r="J6" s="5">
         <v>0</v>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="8">
+    <row r="7" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A7" s="2">
         <v>3</v>
       </c>
-      <c r="B7" s="9" t="s">
+      <c r="B7" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="C7" s="9" t="s">
+      <c r="C7" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="D7" s="10" t="s">
+      <c r="D7" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="E7" s="11">
+      <c r="E7" s="5">
         <v>2178000</v>
       </c>
-      <c r="F7" s="11">
-        <v>0</v>
-      </c>
-      <c r="G7" s="11">
+      <c r="F7" s="5">
+        <v>0</v>
+      </c>
+      <c r="G7" s="5">
         <v>15136264</v>
       </c>
-      <c r="H7" s="9" t="s">
+      <c r="H7" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="I7" s="10" t="s">
+      <c r="I7" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="J7" s="11">
+      <c r="J7" s="5">
         <v>0</v>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="8">
+    <row r="8" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A8" s="2">
         <v>4</v>
       </c>
-      <c r="B8" s="9" t="s">
+      <c r="B8" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="C8" s="9" t="s">
+      <c r="C8" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="D8" s="10" t="s">
+      <c r="D8" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="E8" s="11">
-        <v>0</v>
-      </c>
-      <c r="F8" s="11">
+      <c r="E8" s="5">
+        <v>0</v>
+      </c>
+      <c r="F8" s="5">
         <v>5694170</v>
       </c>
-      <c r="G8" s="11">
+      <c r="G8" s="5">
         <v>17314264</v>
       </c>
-      <c r="H8" s="9" t="s">
+      <c r="H8" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="I8" s="10" t="s">
+      <c r="I8" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="J8" s="11">
+      <c r="J8" s="5">
         <v>0</v>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="8">
+    <row r="9" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A9" s="2">
         <v>5</v>
       </c>
-      <c r="B9" s="9" t="s">
+      <c r="B9" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="C9" s="9" t="s">
+      <c r="C9" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="D9" s="10" t="s">
+      <c r="D9" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="E9" s="11">
+      <c r="E9" s="5">
         <v>107800</v>
       </c>
-      <c r="F9" s="11">
-        <v>0</v>
-      </c>
-      <c r="G9" s="11">
+      <c r="F9" s="5">
+        <v>0</v>
+      </c>
+      <c r="G9" s="5">
         <v>11620094</v>
       </c>
-      <c r="H9" s="9" t="s">
+      <c r="H9" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="I9" s="10" t="s">
+      <c r="I9" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="J9" s="11">
+      <c r="J9" s="5">
         <v>0</v>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="8">
+    <row r="10" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A10" s="2">
         <v>6</v>
       </c>
-      <c r="B10" s="9" t="s">
+      <c r="B10" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="C10" s="9" t="s">
+      <c r="C10" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="D10" s="10" t="s">
+      <c r="D10" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="E10" s="11">
+      <c r="E10" s="5">
         <v>85621</v>
       </c>
-      <c r="F10" s="11">
-        <v>0</v>
-      </c>
-      <c r="G10" s="11">
+      <c r="F10" s="5">
+        <v>0</v>
+      </c>
+      <c r="G10" s="5">
         <v>11727894</v>
       </c>
-      <c r="H10" s="9" t="s">
+      <c r="H10" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="I10" s="10" t="s">
+      <c r="I10" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="J10" s="11">
+      <c r="J10" s="5">
         <v>0</v>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="8">
+    <row r="11" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A11" s="2">
         <v>7</v>
       </c>
-      <c r="B11" s="9" t="s">
+      <c r="B11" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="C11" s="9" t="s">
+      <c r="C11" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="D11" s="10" t="s">
+      <c r="D11" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="E11" s="11">
+      <c r="E11" s="5">
         <v>134622</v>
       </c>
-      <c r="F11" s="11">
-        <v>0</v>
-      </c>
-      <c r="G11" s="11">
+      <c r="F11" s="5">
+        <v>0</v>
+      </c>
+      <c r="G11" s="5">
         <v>11813515</v>
       </c>
-      <c r="H11" s="9" t="s">
+      <c r="H11" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="I11" s="10" t="s">
+      <c r="I11" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="J11" s="11">
+      <c r="J11" s="5">
         <v>0</v>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="8">
+    <row r="12" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A12" s="2">
         <v>8</v>
       </c>
-      <c r="B12" s="9" t="s">
+      <c r="B12" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="C12" s="9" t="s">
+      <c r="C12" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="D12" s="10" t="s">
+      <c r="D12" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="E12" s="11">
-        <v>0</v>
-      </c>
-      <c r="F12" s="11">
+      <c r="E12" s="5">
+        <v>0</v>
+      </c>
+      <c r="F12" s="5">
         <v>2852</v>
       </c>
-      <c r="G12" s="11">
+      <c r="G12" s="5">
         <v>11948137</v>
       </c>
-      <c r="H12" s="9" t="s">
+      <c r="H12" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="I12" s="10" t="s">
+      <c r="I12" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="J12" s="11">
+      <c r="J12" s="5">
         <v>0</v>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="10" t="s">
+    <row r="13" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A13" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="B13" s="9" t="s">
+      <c r="B13" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="C13" s="10" t="s">
+      <c r="C13" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="D13" s="10" t="s">
+      <c r="D13" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="E13" s="12" t="s">
+      <c r="E13" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="F13" s="12" t="s">
+      <c r="F13" s="6" t="s">
         <v>38</v>
       </c>
-      <c r="G13" s="11">
-        <v>0</v>
-      </c>
-      <c r="H13" s="10" t="s">
+      <c r="G13" s="5">
+        <v>0</v>
+      </c>
+      <c r="H13" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="I13" s="10" t="s">
+      <c r="I13" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="J13" s="11">
+      <c r="J13" s="5">
         <v>0</v>
       </c>
     </row>
@@ -1211,5 +1223,7 @@
     <mergeCell ref="A2:J2"/>
     <mergeCell ref="A3:J3"/>
   </mergeCells>
+  <phoneticPr fontId="11" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>